<commit_message>
fix: align IATF export template output
</commit_message>
<xml_diff>
--- a/sheet_cutting_layout/templates/iatf/sheet_cutting_layout.xlsx
+++ b/sheet_cutting_layout/templates/iatf/sheet_cutting_layout.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="61">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -85,7 +85,7 @@
     <t>Sheet size (Width x Length)</t>
   </si>
   <si>
-    <t>END PIECE</t>
+    <t>END PIECE 1</t>
   </si>
   <si>
     <t>Weight of Strip</t>
@@ -94,45 +94,51 @@
     <t>kgs</t>
   </si>
   <si>
+    <t>END PIECE 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Strip Size:-                                                   </t>
   </si>
   <si>
+    <t>END PIECE 3</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part Per Strip:-                                          </t>
   </si>
   <si>
     <t>Nos</t>
   </si>
   <si>
+    <t>No. of strips</t>
+  </si>
+  <si>
     <t>II</t>
   </si>
   <si>
     <t xml:space="preserve">End Piece 2 Size :-                                      </t>
   </si>
   <si>
-    <t>No. of strips</t>
+    <t xml:space="preserve">Part Per Sheet:-                                         </t>
   </si>
   <si>
     <t>Used For Part Number:-</t>
   </si>
   <si>
-    <t xml:space="preserve">Part Per Sheet:-                                         </t>
+    <t xml:space="preserve">Gross Weight of a part:-                        </t>
+  </si>
+  <si>
+    <t>kg</t>
   </si>
   <si>
     <t xml:space="preserve">Strip Size(Width x Length):-                                                   </t>
   </si>
   <si>
-    <t xml:space="preserve">Gross Weight of a part:-                        </t>
-  </si>
-  <si>
-    <t>kg</t>
+    <t xml:space="preserve">Net Wt. of a finished Part:-                                 </t>
   </si>
   <si>
     <t xml:space="preserve">Part Per Strip:-                                         </t>
   </si>
   <si>
-    <t xml:space="preserve">Net Wt. of a finished Part:-                                 </t>
-  </si>
-  <si>
     <t xml:space="preserve">Scrap Weight of a Part:-                           </t>
   </si>
   <si>
@@ -142,13 +148,13 @@
     <t xml:space="preserve">End Piece 1 Size :-                                     </t>
   </si>
   <si>
+    <t>III</t>
+  </si>
+  <si>
+    <t xml:space="preserve">End Piece 3 Size :-                                      </t>
+  </si>
+  <si>
     <t>End Piece 2-A Size :-</t>
-  </si>
-  <si>
-    <t>III</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End Piece 3 Size :-                                      </t>
   </si>
   <si>
     <t>End Piece 2-B Size :-</t>
@@ -250,7 +256,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -263,14 +269,8 @@
         <bgColor theme="0"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFFC000"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="53">
+  <borders count="56">
     <border/>
     <border>
       <left style="medium">
@@ -559,7 +559,7 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color rgb="FF000000"/>
       </left>
       <bottom style="thin">
@@ -639,6 +639,17 @@
       </bottom>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -653,6 +664,56 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
       <top style="medium">
         <color rgb="FF000000"/>
       </top>
@@ -697,9 +758,6 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -708,31 +766,6 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -749,20 +782,20 @@
       </top>
     </border>
     <border>
-      <left style="medium">
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FF000000"/>
       </left>
       <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
     </border>
@@ -880,10 +913,10 @@
     <xf borderId="39" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="40" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="40" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="41" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="38" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
@@ -896,8 +929,8 @@
     <xf borderId="39" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf borderId="40" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="38" fillId="0" fontId="6" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
@@ -909,16 +942,29 @@
     <xf borderId="39" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="42" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="43" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="44" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="44" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="45" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="38" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="39" fillId="0" fontId="5" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="36" fillId="0" fontId="5" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="38" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="41" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="46" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -930,10 +976,10 @@
     <xf borderId="32" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="42" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="47" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="43" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="48" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="11" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -942,26 +988,20 @@
     <xf borderId="11" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="43" fillId="0" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="48" fillId="0" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="2" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="168" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="38" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="38" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="39" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="39" fillId="0" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="11" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="38" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="39" fillId="0" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
@@ -971,13 +1011,6 @@
     <xf borderId="11" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="38" fillId="3" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="39" fillId="3" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="37" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -987,9 +1020,25 @@
     <xf borderId="38" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="38" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="49" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="44" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="44" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="44" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="45" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="11" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -999,36 +1048,18 @@
     <xf borderId="39" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="44" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="49" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="50" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="50" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="45" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="45" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="45" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="46" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="44" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="47" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="45" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="47" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="46" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="31" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1038,7 +1069,7 @@
     <xf borderId="32" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="42" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="47" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1057,21 +1088,21 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="43" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="45" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="48" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="44" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="48" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="51" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="49" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="50" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="51" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="52" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="33" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="53" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="24" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="52" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="54" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1081,8 +1112,8 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="33" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="51" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="55" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="53" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1111,34 +1142,6 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="3009900" cy="4352925"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1633,14 +1636,14 @@
       </c>
       <c r="P9" s="52"/>
       <c r="Q9" s="53">
-        <f>+K27</f>
+        <f>+K28</f>
         <v>3.96144</v>
       </c>
       <c r="R9" s="53">
         <v>0.0</v>
       </c>
       <c r="S9" s="58" t="str">
-        <f>K28</f>
+        <f>K29</f>
         <v/>
       </c>
       <c r="T9" s="55">
@@ -1673,26 +1676,26 @@
       <c r="M10" s="61"/>
       <c r="N10" s="40"/>
       <c r="O10" s="57" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P10" s="52"/>
       <c r="Q10" s="53">
-        <f>R16+R26</f>
+        <f t="shared" ref="Q10:Q11" si="1">R17+R27</f>
         <v>0</v>
       </c>
       <c r="R10" s="53" t="str">
-        <f>R17</f>
+        <f t="shared" ref="R10:R11" si="2">R18</f>
         <v/>
       </c>
       <c r="S10" s="53" t="str">
-        <f>R18</f>
+        <f t="shared" ref="S10:S11" si="3">R19</f>
         <v/>
       </c>
       <c r="T10" s="55">
         <v>1.0</v>
       </c>
       <c r="U10" s="56">
-        <f>T10*Q10</f>
+        <f t="shared" ref="U10:U11" si="4">T10*Q10</f>
         <v>0</v>
       </c>
     </row>
@@ -1704,7 +1707,7 @@
         <v>5.0</v>
       </c>
       <c r="I11" s="47" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J11" s="48" t="s">
         <v>21</v>
@@ -1719,15 +1722,28 @@
         <v>281.0</v>
       </c>
       <c r="N11" s="40"/>
-      <c r="O11" s="62"/>
-      <c r="P11" s="62"/>
-      <c r="Q11" s="40"/>
-      <c r="R11" s="40"/>
-      <c r="S11" s="40"/>
-      <c r="T11" s="40"/>
-      <c r="U11" s="63">
-        <f>SUM(U8:U10)</f>
-        <v>39.3</v>
+      <c r="O11" s="62" t="s">
+        <v>29</v>
+      </c>
+      <c r="P11" s="63"/>
+      <c r="Q11" s="64">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="R11" s="64" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="S11" s="64" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="T11" s="65">
+        <v>1.0</v>
+      </c>
+      <c r="U11" s="66">
+        <f t="shared" si="4"/>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1738,39 +1754,27 @@
         <v>6.0</v>
       </c>
       <c r="I12" s="47" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J12" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="K12" s="64">
+        <v>31</v>
+      </c>
+      <c r="K12" s="67">
         <v>6.0</v>
       </c>
       <c r="L12" s="48"/>
       <c r="M12" s="50"/>
       <c r="N12" s="40"/>
-      <c r="O12" s="65" t="s">
-        <v>30</v>
-      </c>
-      <c r="P12" s="66" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q12" s="67" t="s">
-        <v>21</v>
-      </c>
-      <c r="R12" s="68" t="str">
-        <f t="shared" ref="R12:T12" si="1">K19</f>
-        <v/>
-      </c>
-      <c r="S12" s="68" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="T12" s="69" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="U12" s="70"/>
+      <c r="O12" s="68"/>
+      <c r="P12" s="68"/>
+      <c r="Q12" s="40"/>
+      <c r="R12" s="40"/>
+      <c r="S12" s="40"/>
+      <c r="T12" s="40"/>
+      <c r="U12" s="69">
+        <f>SUM(U8:U11)</f>
+        <v>39.3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="45"/>
@@ -1783,27 +1787,36 @@
         <v>32</v>
       </c>
       <c r="J13" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="K13" s="64">
+        <v>31</v>
+      </c>
+      <c r="K13" s="67">
         <v>8.0</v>
       </c>
       <c r="L13" s="48"/>
       <c r="M13" s="50"/>
       <c r="N13" s="40"/>
-      <c r="O13" s="46">
-        <v>1.0</v>
+      <c r="O13" s="70" t="s">
+        <v>33</v>
       </c>
       <c r="P13" s="71" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q13" s="72"/>
-      <c r="R13" s="13"/>
-      <c r="S13" s="13"/>
-      <c r="T13" s="14"/>
-      <c r="U13" s="73"/>
-      <c r="W13" s="74"/>
-      <c r="X13" s="75"/>
+        <v>34</v>
+      </c>
+      <c r="Q13" s="72" t="s">
+        <v>21</v>
+      </c>
+      <c r="R13" s="73" t="str">
+        <f t="shared" ref="R13:T13" si="5">K19</f>
+        <v/>
+      </c>
+      <c r="S13" s="73" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="T13" s="74" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="U13" s="75"/>
     </row>
     <row r="14">
       <c r="A14" s="45"/>
@@ -1813,42 +1826,31 @@
         <v>8.0</v>
       </c>
       <c r="I14" s="47" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J14" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="K14" s="76">
+        <v>31</v>
+      </c>
+      <c r="K14" s="48">
         <f>+K13*K12</f>
         <v>48</v>
       </c>
-      <c r="L14" s="76"/>
-      <c r="M14" s="77"/>
+      <c r="L14" s="48"/>
+      <c r="M14" s="50"/>
       <c r="N14" s="40"/>
       <c r="O14" s="46">
-        <v>2.0</v>
-      </c>
-      <c r="P14" s="71" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q14" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="R14" s="78" t="str">
-        <f t="shared" ref="R14:T14" si="2">R12</f>
-        <v/>
-      </c>
-      <c r="S14" s="78" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="T14" s="50" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="U14" s="70"/>
-      <c r="W14" s="27"/>
-      <c r="X14" s="27"/>
+        <v>1.0</v>
+      </c>
+      <c r="P14" s="76" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q14" s="77"/>
+      <c r="R14" s="13"/>
+      <c r="S14" s="13"/>
+      <c r="T14" s="14"/>
+      <c r="U14" s="78"/>
+      <c r="W14" s="79"/>
+      <c r="X14" s="80"/>
     </row>
     <row r="15">
       <c r="A15" s="45"/>
@@ -1858,32 +1860,41 @@
         <v>9.0</v>
       </c>
       <c r="I15" s="47" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J15" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="K15" s="79">
+        <v>38</v>
+      </c>
+      <c r="K15" s="81">
         <f>+(K10/K12)</f>
         <v>0.73622</v>
       </c>
       <c r="L15" s="60"/>
-      <c r="M15" s="80"/>
+      <c r="M15" s="82"/>
       <c r="N15" s="40"/>
       <c r="O15" s="46">
-        <v>3.0</v>
-      </c>
-      <c r="P15" s="71" t="s">
-        <v>38</v>
+        <v>2.0</v>
+      </c>
+      <c r="P15" s="76" t="s">
+        <v>39</v>
       </c>
       <c r="Q15" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="R15" s="78"/>
-      <c r="S15" s="13"/>
-      <c r="T15" s="14"/>
-      <c r="U15" s="70"/>
-      <c r="W15" s="81"/>
+        <v>21</v>
+      </c>
+      <c r="R15" s="83" t="str">
+        <f t="shared" ref="R15:T15" si="6">R13</f>
+        <v/>
+      </c>
+      <c r="S15" s="83" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="T15" s="50" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="U15" s="75"/>
+      <c r="W15" s="27"/>
       <c r="X15" s="27"/>
     </row>
     <row r="16">
@@ -1894,34 +1905,31 @@
         <v>10.0</v>
       </c>
       <c r="I16" s="47" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J16" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="K16" s="79">
+        <v>38</v>
+      </c>
+      <c r="K16" s="81">
         <v>0.292</v>
       </c>
       <c r="L16" s="48"/>
       <c r="M16" s="50"/>
       <c r="N16" s="40"/>
       <c r="O16" s="46">
-        <v>4.0</v>
-      </c>
-      <c r="P16" s="71" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q16" s="82" t="s">
-        <v>37</v>
-      </c>
-      <c r="R16" s="83">
-        <f>+R14*S14*T14*0.786/100000</f>
-        <v>0</v>
-      </c>
+        <v>3.0</v>
+      </c>
+      <c r="P16" s="76" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q16" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="R16" s="83"/>
       <c r="S16" s="13"/>
       <c r="T16" s="14"/>
-      <c r="U16" s="70"/>
-      <c r="W16" s="27"/>
+      <c r="U16" s="75"/>
+      <c r="W16" s="84"/>
       <c r="X16" s="27"/>
     </row>
     <row r="17">
@@ -1932,34 +1940,34 @@
         <v>11.0</v>
       </c>
       <c r="I17" s="47" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J17" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="K17" s="84">
+        <v>38</v>
+      </c>
+      <c r="K17" s="60">
         <f>+K15-K16</f>
         <v>0.44422</v>
       </c>
-      <c r="L17" s="84"/>
-      <c r="M17" s="85"/>
+      <c r="L17" s="60"/>
+      <c r="M17" s="82"/>
       <c r="N17" s="40"/>
       <c r="O17" s="46">
-        <v>5.0</v>
-      </c>
-      <c r="P17" s="71" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q17" s="48" t="s">
+        <v>4.0</v>
+      </c>
+      <c r="P17" s="76" t="s">
         <v>37</v>
       </c>
-      <c r="R17" s="83"/>
+      <c r="Q17" s="85" t="s">
+        <v>38</v>
+      </c>
+      <c r="R17" s="86">
+        <f>+R15*S15*T15*0.786/100000</f>
+        <v>0</v>
+      </c>
       <c r="S17" s="13"/>
       <c r="T17" s="14"/>
-      <c r="U17" s="70"/>
-      <c r="V17" s="86" t="s">
-        <v>0</v>
-      </c>
+      <c r="U17" s="75"/>
       <c r="W17" s="27"/>
       <c r="X17" s="27"/>
     </row>
@@ -1968,10 +1976,10 @@
       <c r="F18" s="11"/>
       <c r="G18" s="29"/>
       <c r="H18" s="87" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I18" s="88" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J18" s="89" t="s">
         <v>21</v>
@@ -1988,18 +1996,21 @@
       </c>
       <c r="N18" s="40"/>
       <c r="O18" s="46">
-        <v>6.0</v>
-      </c>
-      <c r="P18" s="71" t="s">
+        <v>5.0</v>
+      </c>
+      <c r="P18" s="76" t="s">
         <v>40</v>
       </c>
       <c r="Q18" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="R18" s="83"/>
+        <v>38</v>
+      </c>
+      <c r="R18" s="86"/>
       <c r="S18" s="13"/>
       <c r="T18" s="14"/>
-      <c r="U18" s="70"/>
+      <c r="U18" s="75"/>
+      <c r="V18" s="90" t="s">
+        <v>0</v>
+      </c>
       <c r="W18" s="27"/>
       <c r="X18" s="27"/>
     </row>
@@ -2008,31 +2019,31 @@
       <c r="F19" s="11"/>
       <c r="G19" s="29"/>
       <c r="H19" s="87" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I19" s="88" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J19" s="89" t="s">
         <v>21</v>
       </c>
       <c r="K19" s="48"/>
-      <c r="L19" s="90"/>
+      <c r="L19" s="91"/>
       <c r="M19" s="50"/>
       <c r="N19" s="40"/>
       <c r="O19" s="46">
-        <v>7.0</v>
-      </c>
-      <c r="P19" s="91" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q19" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="R19" s="92"/>
-      <c r="S19" s="92"/>
-      <c r="T19" s="93"/>
-      <c r="U19" s="70"/>
+        <v>6.0</v>
+      </c>
+      <c r="P19" s="76" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q19" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19" s="86"/>
+      <c r="S19" s="13"/>
+      <c r="T19" s="14"/>
+      <c r="U19" s="75"/>
       <c r="W19" s="27"/>
       <c r="X19" s="27"/>
     </row>
@@ -2040,53 +2051,53 @@
       <c r="A20" s="45"/>
       <c r="F20" s="11"/>
       <c r="G20" s="29"/>
-      <c r="H20" s="94" t="s">
-        <v>44</v>
-      </c>
-      <c r="I20" s="95" t="s">
+      <c r="H20" s="92" t="s">
         <v>45</v>
       </c>
-      <c r="J20" s="96" t="s">
+      <c r="I20" s="93" t="s">
+        <v>46</v>
+      </c>
+      <c r="J20" s="94" t="s">
         <v>21</v>
       </c>
-      <c r="K20" s="48"/>
-      <c r="L20" s="97"/>
-      <c r="M20" s="98"/>
+      <c r="K20" s="95"/>
+      <c r="L20" s="95"/>
+      <c r="M20" s="96"/>
       <c r="N20" s="40"/>
-      <c r="O20" s="99">
-        <v>8.0</v>
-      </c>
-      <c r="P20" s="100" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q20" s="101" t="s">
+      <c r="O20" s="46">
+        <v>7.0</v>
+      </c>
+      <c r="P20" s="97" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q20" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="R20" s="102"/>
-      <c r="S20" s="102"/>
-      <c r="T20" s="103"/>
-      <c r="U20" s="70"/>
+      <c r="R20" s="98"/>
+      <c r="S20" s="98"/>
+      <c r="T20" s="99"/>
+      <c r="U20" s="75"/>
       <c r="W20" s="27"/>
       <c r="X20" s="27"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21">
       <c r="A21" s="45"/>
       <c r="F21" s="11"/>
       <c r="G21" s="29"/>
-      <c r="H21" s="62"/>
-      <c r="I21" s="40"/>
-      <c r="J21" s="40"/>
-      <c r="K21" s="40"/>
-      <c r="L21" s="40"/>
-      <c r="M21" s="40"/>
       <c r="N21" s="40"/>
-      <c r="O21" s="27"/>
-      <c r="P21" s="27"/>
-      <c r="Q21" s="27"/>
-      <c r="R21" s="27"/>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
-      <c r="U21" s="70"/>
+      <c r="O21" s="100">
+        <v>8.0</v>
+      </c>
+      <c r="P21" s="101" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q21" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="R21" s="102"/>
+      <c r="S21" s="102"/>
+      <c r="T21" s="103"/>
+      <c r="U21" s="75"/>
       <c r="W21" s="27"/>
       <c r="X21" s="27"/>
     </row>
@@ -2094,80 +2105,72 @@
       <c r="A22" s="45"/>
       <c r="F22" s="11"/>
       <c r="G22" s="29"/>
-      <c r="H22" s="104" t="s">
-        <v>41</v>
-      </c>
-      <c r="I22" s="105" t="s">
-        <v>47</v>
-      </c>
-      <c r="J22" s="67" t="s">
-        <v>21</v>
-      </c>
-      <c r="K22" s="106">
-        <f t="shared" ref="K22:M22" si="3">+K18</f>
-        <v>1.6</v>
-      </c>
-      <c r="L22" s="67">
-        <f t="shared" si="3"/>
-        <v>252</v>
-      </c>
-      <c r="M22" s="107">
-        <f t="shared" si="3"/>
-        <v>1250</v>
-      </c>
+      <c r="H22" s="68"/>
+      <c r="I22" s="40"/>
+      <c r="J22" s="40"/>
+      <c r="K22" s="40"/>
+      <c r="L22" s="40"/>
+      <c r="M22" s="40"/>
       <c r="N22" s="40"/>
-      <c r="O22" s="104" t="s">
-        <v>44</v>
-      </c>
-      <c r="P22" s="108" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q22" s="67" t="s">
-        <v>21</v>
-      </c>
-      <c r="R22" s="67" t="str">
-        <f t="shared" ref="R22:T22" si="4">K20</f>
-        <v/>
-      </c>
-      <c r="S22" s="67" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="T22" s="67" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="U22" s="70"/>
-      <c r="W22" s="109"/>
+      <c r="O22" s="27"/>
+      <c r="P22" s="27"/>
+      <c r="Q22" s="27"/>
+      <c r="R22" s="27"/>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="75"/>
+      <c r="W22" s="27"/>
       <c r="X22" s="27"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="45"/>
       <c r="F23" s="11"/>
       <c r="G23" s="29"/>
-      <c r="H23" s="46">
-        <v>1.0</v>
-      </c>
-      <c r="I23" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="J23" s="78"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="14"/>
+      <c r="H23" s="104" t="s">
+        <v>43</v>
+      </c>
+      <c r="I23" s="105" t="s">
+        <v>49</v>
+      </c>
+      <c r="J23" s="72" t="s">
+        <v>21</v>
+      </c>
+      <c r="K23" s="106">
+        <f t="shared" ref="K23:M23" si="7">+K18</f>
+        <v>1.6</v>
+      </c>
+      <c r="L23" s="72">
+        <f t="shared" si="7"/>
+        <v>252</v>
+      </c>
+      <c r="M23" s="107">
+        <f t="shared" si="7"/>
+        <v>1250</v>
+      </c>
       <c r="N23" s="40"/>
-      <c r="O23" s="46">
-        <v>1.0</v>
-      </c>
-      <c r="P23" s="71" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q23" s="78"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-      <c r="T23" s="14"/>
-      <c r="U23" s="70"/>
-      <c r="W23" s="27"/>
+      <c r="O23" s="104" t="s">
+        <v>45</v>
+      </c>
+      <c r="P23" s="108" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q23" s="72" t="s">
+        <v>21</v>
+      </c>
+      <c r="R23" s="72" t="str">
+        <f t="shared" ref="R23:T23" si="8">K20</f>
+        <v/>
+      </c>
+      <c r="S23" s="72" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="T23" s="72" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="U23" s="75"/>
+      <c r="W23" s="109"/>
       <c r="X23" s="27"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -2175,49 +2178,27 @@
       <c r="F24" s="11"/>
       <c r="G24" s="29"/>
       <c r="H24" s="46">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="I24" s="47" t="s">
-        <v>35</v>
-      </c>
-      <c r="J24" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="K24" s="49">
-        <f t="shared" ref="K24:M24" si="5">+K22</f>
-        <v>1.6</v>
-      </c>
-      <c r="L24" s="48">
-        <f t="shared" si="5"/>
-        <v>252</v>
-      </c>
-      <c r="M24" s="50">
-        <f t="shared" si="5"/>
-        <v>1250</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="J24" s="83"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="14"/>
       <c r="N24" s="40"/>
       <c r="O24" s="46">
-        <v>2.0</v>
-      </c>
-      <c r="P24" s="71" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q24" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="R24" s="78" t="str">
-        <f t="shared" ref="R24:T24" si="6">+R22</f>
-        <v/>
-      </c>
-      <c r="S24" s="78" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="T24" s="110" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="U24" s="70"/>
+        <v>1.0</v>
+      </c>
+      <c r="P24" s="76" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q24" s="83"/>
+      <c r="R24" s="13"/>
+      <c r="S24" s="13"/>
+      <c r="T24" s="14"/>
+      <c r="U24" s="75"/>
       <c r="W24" s="27"/>
       <c r="X24" s="27"/>
     </row>
@@ -2226,31 +2207,49 @@
       <c r="F25" s="11"/>
       <c r="G25" s="29"/>
       <c r="H25" s="46">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="I25" s="47" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="J25" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="K25" s="48"/>
-      <c r="L25" s="48"/>
-      <c r="M25" s="50"/>
+        <v>21</v>
+      </c>
+      <c r="K25" s="49">
+        <f t="shared" ref="K25:M25" si="9">+K23</f>
+        <v>1.6</v>
+      </c>
+      <c r="L25" s="48">
+        <f t="shared" si="9"/>
+        <v>252</v>
+      </c>
+      <c r="M25" s="50">
+        <f t="shared" si="9"/>
+        <v>1250</v>
+      </c>
       <c r="N25" s="40"/>
       <c r="O25" s="46">
-        <v>3.0</v>
-      </c>
-      <c r="P25" s="71" t="s">
-        <v>28</v>
+        <v>2.0</v>
+      </c>
+      <c r="P25" s="76" t="s">
+        <v>39</v>
       </c>
       <c r="Q25" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="R25" s="78"/>
-      <c r="S25" s="13"/>
-      <c r="T25" s="14"/>
-      <c r="U25" s="70"/>
+        <v>21</v>
+      </c>
+      <c r="R25" s="83" t="str">
+        <f t="shared" ref="R25:T25" si="10">+R23</f>
+        <v/>
+      </c>
+      <c r="S25" s="83" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="T25" s="110" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="U25" s="75"/>
       <c r="W25" s="27"/>
       <c r="X25" s="27"/>
     </row>
@@ -2259,34 +2258,31 @@
       <c r="F26" s="11"/>
       <c r="G26" s="29"/>
       <c r="H26" s="46">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="I26" s="47" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="J26" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="K26" s="79"/>
-      <c r="L26" s="48"/>
-      <c r="M26" s="50"/>
+        <v>31</v>
+      </c>
+      <c r="K26" s="83"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="14"/>
       <c r="N26" s="40"/>
       <c r="O26" s="46">
-        <v>4.0</v>
-      </c>
-      <c r="P26" s="71" t="s">
-        <v>36</v>
+        <v>3.0</v>
+      </c>
+      <c r="P26" s="76" t="s">
+        <v>30</v>
       </c>
       <c r="Q26" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="R26" s="83">
-        <f>+R24*S24*T24*0.786/100000</f>
-        <v>0</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="R26" s="83"/>
       <c r="S26" s="13"/>
       <c r="T26" s="14"/>
-      <c r="U26" s="70"/>
+      <c r="U26" s="75"/>
       <c r="W26" s="27"/>
       <c r="X26" s="27"/>
     </row>
@@ -2295,334 +2291,369 @@
       <c r="F27" s="11"/>
       <c r="G27" s="29"/>
       <c r="H27" s="46">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="I27" s="47" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J27" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="K27" s="83">
-        <f>+K24*L24*M24*0.786/100000</f>
-        <v>3.96144</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="K27" s="86"/>
       <c r="L27" s="13"/>
       <c r="M27" s="14"/>
       <c r="N27" s="40"/>
       <c r="O27" s="46">
-        <v>5.0</v>
-      </c>
-      <c r="P27" s="71" t="s">
-        <v>39</v>
+        <v>4.0</v>
+      </c>
+      <c r="P27" s="76" t="s">
+        <v>37</v>
       </c>
       <c r="Q27" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="R27" s="78"/>
+        <v>38</v>
+      </c>
+      <c r="R27" s="86">
+        <f>+R25*S25*T25*0.786/100000</f>
+        <v>0</v>
+      </c>
       <c r="S27" s="13"/>
       <c r="T27" s="14"/>
-      <c r="U27" s="70"/>
+      <c r="U27" s="75"/>
       <c r="W27" s="27"/>
       <c r="X27" s="27"/>
-      <c r="Z27" s="111"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="45"/>
       <c r="F28" s="11"/>
       <c r="G28" s="29"/>
       <c r="H28" s="46">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="I28" s="47" t="s">
         <v>40</v>
       </c>
       <c r="J28" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="K28" s="83"/>
+        <v>38</v>
+      </c>
+      <c r="K28" s="86">
+        <f>+K25*L25*M25*0.786/100000</f>
+        <v>3.96144</v>
+      </c>
       <c r="L28" s="13"/>
       <c r="M28" s="14"/>
       <c r="N28" s="40"/>
       <c r="O28" s="46">
-        <v>6.0</v>
-      </c>
-      <c r="P28" s="71" t="s">
+        <v>5.0</v>
+      </c>
+      <c r="P28" s="76" t="s">
         <v>40</v>
       </c>
       <c r="Q28" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="R28" s="78"/>
+        <v>38</v>
+      </c>
+      <c r="R28" s="83"/>
       <c r="S28" s="13"/>
       <c r="T28" s="14"/>
-      <c r="U28" s="70"/>
+      <c r="U28" s="75"/>
       <c r="W28" s="27"/>
       <c r="X28" s="27"/>
+      <c r="Z28" s="111"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="45"/>
       <c r="F29" s="11"/>
       <c r="G29" s="29"/>
       <c r="H29" s="46">
-        <v>7.0</v>
-      </c>
-      <c r="I29" s="112" t="s">
-        <v>48</v>
-      </c>
-      <c r="J29" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="K29" s="92"/>
-      <c r="L29" s="92"/>
-      <c r="M29" s="93"/>
-      <c r="N29" s="113"/>
+        <v>6.0</v>
+      </c>
+      <c r="I29" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="J29" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="K29" s="86"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="14"/>
+      <c r="N29" s="40"/>
       <c r="O29" s="46">
-        <v>7.0</v>
-      </c>
-      <c r="P29" s="91" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q29" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="R29" s="92"/>
-      <c r="S29" s="92"/>
-      <c r="T29" s="93"/>
-      <c r="U29" s="114"/>
+        <v>6.0</v>
+      </c>
+      <c r="P29" s="76" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q29" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="R29" s="83"/>
+      <c r="S29" s="13"/>
+      <c r="T29" s="14"/>
+      <c r="U29" s="75"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="27"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="45"/>
       <c r="F30" s="11"/>
       <c r="G30" s="29"/>
-      <c r="H30" s="99">
-        <v>8.0</v>
-      </c>
-      <c r="I30" s="115" t="s">
+      <c r="H30" s="46">
+        <v>7.0</v>
+      </c>
+      <c r="I30" s="112" t="s">
         <v>50</v>
       </c>
-      <c r="J30" s="101" t="s">
+      <c r="J30" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="K30" s="102"/>
-      <c r="L30" s="102"/>
-      <c r="M30" s="103"/>
+      <c r="K30" s="98"/>
+      <c r="L30" s="98"/>
+      <c r="M30" s="99"/>
       <c r="N30" s="113"/>
-      <c r="O30" s="99">
-        <v>8.0</v>
-      </c>
-      <c r="P30" s="100" t="s">
+      <c r="O30" s="46">
+        <v>7.0</v>
+      </c>
+      <c r="P30" s="97" t="s">
         <v>51</v>
       </c>
-      <c r="Q30" s="101" t="s">
+      <c r="Q30" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="R30" s="102"/>
-      <c r="S30" s="102"/>
-      <c r="T30" s="103"/>
+      <c r="R30" s="98"/>
+      <c r="S30" s="98"/>
+      <c r="T30" s="99"/>
       <c r="U30" s="114"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="45"/>
       <c r="F31" s="11"/>
       <c r="G31" s="29"/>
-      <c r="H31" s="62"/>
-      <c r="I31" s="116"/>
-      <c r="J31" s="116"/>
-      <c r="K31" s="116"/>
-      <c r="L31" s="116"/>
-      <c r="M31" s="116"/>
-      <c r="N31" s="116"/>
-      <c r="O31" s="116"/>
-      <c r="P31" s="116"/>
-      <c r="Q31" s="27"/>
-      <c r="R31" s="27"/>
-      <c r="S31" s="27"/>
-      <c r="T31" s="27"/>
+      <c r="H31" s="100">
+        <v>8.0</v>
+      </c>
+      <c r="I31" s="115" t="s">
+        <v>52</v>
+      </c>
+      <c r="J31" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="K31" s="102"/>
+      <c r="L31" s="102"/>
+      <c r="M31" s="103"/>
+      <c r="N31" s="113"/>
+      <c r="O31" s="100">
+        <v>8.0</v>
+      </c>
+      <c r="P31" s="101" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q31" s="65" t="s">
+        <v>21</v>
+      </c>
+      <c r="R31" s="102"/>
+      <c r="S31" s="102"/>
+      <c r="T31" s="103"/>
       <c r="U31" s="114"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="45"/>
       <c r="F32" s="11"/>
       <c r="G32" s="29"/>
-      <c r="H32" s="117" t="s">
-        <v>52</v>
-      </c>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
-      <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
-      <c r="N32" s="3"/>
-      <c r="O32" s="3"/>
-      <c r="P32" s="3"/>
-      <c r="Q32" s="3"/>
-      <c r="R32" s="3"/>
-      <c r="S32" s="3"/>
-      <c r="T32" s="118"/>
+      <c r="H32" s="68"/>
+      <c r="I32" s="116"/>
+      <c r="J32" s="116"/>
+      <c r="K32" s="116"/>
+      <c r="L32" s="116"/>
+      <c r="M32" s="116"/>
+      <c r="N32" s="116"/>
+      <c r="O32" s="116"/>
+      <c r="P32" s="116"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
       <c r="U32" s="114"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="119"/>
-      <c r="B33" s="120"/>
-      <c r="C33" s="120"/>
-      <c r="D33" s="120"/>
-      <c r="E33" s="120"/>
-      <c r="F33" s="42"/>
+      <c r="A33" s="45"/>
+      <c r="F33" s="11"/>
       <c r="G33" s="29"/>
-      <c r="H33" s="121"/>
-      <c r="I33" s="122"/>
-      <c r="J33" s="122"/>
-      <c r="K33" s="122"/>
-      <c r="L33" s="122"/>
-      <c r="M33" s="122"/>
-      <c r="N33" s="122"/>
-      <c r="O33" s="122"/>
-      <c r="P33" s="122"/>
-      <c r="Q33" s="122"/>
-      <c r="R33" s="122"/>
-      <c r="S33" s="122"/>
-      <c r="T33" s="34"/>
+      <c r="H33" s="117" t="s">
+        <v>54</v>
+      </c>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+      <c r="P33" s="3"/>
+      <c r="Q33" s="3"/>
+      <c r="R33" s="3"/>
+      <c r="S33" s="3"/>
+      <c r="T33" s="118"/>
       <c r="U33" s="114"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="26"/>
-      <c r="B34" s="27"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
+      <c r="A34" s="119"/>
+      <c r="B34" s="120"/>
+      <c r="C34" s="120"/>
+      <c r="D34" s="120"/>
+      <c r="E34" s="120"/>
+      <c r="F34" s="42"/>
       <c r="G34" s="29"/>
-      <c r="H34" s="123"/>
-      <c r="I34" s="123"/>
-      <c r="J34" s="123"/>
-      <c r="K34" s="123"/>
-      <c r="L34" s="123"/>
-      <c r="M34" s="123"/>
-      <c r="N34" s="123"/>
-      <c r="O34" s="123"/>
-      <c r="P34" s="123"/>
-      <c r="Q34" s="123"/>
-      <c r="R34" s="123"/>
-      <c r="S34" s="123"/>
-      <c r="T34" s="123"/>
+      <c r="H34" s="121"/>
+      <c r="I34" s="122"/>
+      <c r="J34" s="122"/>
+      <c r="K34" s="122"/>
+      <c r="L34" s="122"/>
+      <c r="M34" s="122"/>
+      <c r="N34" s="122"/>
+      <c r="O34" s="122"/>
+      <c r="P34" s="122"/>
+      <c r="Q34" s="122"/>
+      <c r="R34" s="122"/>
+      <c r="S34" s="122"/>
+      <c r="T34" s="34"/>
       <c r="U34" s="114"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="26"/>
-      <c r="B35" s="113" t="s">
-        <v>53</v>
-      </c>
-      <c r="C35" s="123"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="123"/>
+      <c r="I35" s="123"/>
+      <c r="J35" s="123"/>
+      <c r="K35" s="123"/>
+      <c r="L35" s="123"/>
+      <c r="M35" s="123"/>
+      <c r="N35" s="123"/>
+      <c r="O35" s="123"/>
+      <c r="P35" s="123"/>
+      <c r="Q35" s="123"/>
+      <c r="R35" s="123"/>
+      <c r="S35" s="123"/>
+      <c r="T35" s="123"/>
       <c r="U35" s="114"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="26"/>
-      <c r="B36" s="113"/>
-      <c r="C36" s="113"/>
-      <c r="D36" s="113"/>
-      <c r="E36" s="27"/>
-      <c r="F36" s="27"/>
-      <c r="G36" s="29"/>
-      <c r="H36" s="123"/>
-      <c r="I36" s="123"/>
-      <c r="J36" s="123"/>
-      <c r="K36" s="123"/>
-      <c r="L36" s="123"/>
-      <c r="M36" s="123"/>
-      <c r="N36" s="123"/>
-      <c r="O36" s="123"/>
-      <c r="P36" s="123"/>
-      <c r="Q36" s="123"/>
-      <c r="R36" s="123"/>
-      <c r="S36" s="123"/>
-      <c r="T36" s="123"/>
+      <c r="B36" s="113" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="123"/>
       <c r="U36" s="114"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="26"/>
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
+      <c r="B37" s="113"/>
+      <c r="C37" s="113"/>
+      <c r="D37" s="113"/>
       <c r="E37" s="27"/>
       <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="27"/>
-      <c r="M37" s="27"/>
-      <c r="N37" s="27"/>
-      <c r="O37" s="27"/>
-      <c r="P37" s="27"/>
-      <c r="Q37" s="27"/>
-      <c r="R37" s="27"/>
-      <c r="S37" s="27"/>
-      <c r="T37" s="27"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="123"/>
+      <c r="I37" s="123"/>
+      <c r="J37" s="123"/>
+      <c r="K37" s="123"/>
+      <c r="L37" s="123"/>
+      <c r="M37" s="123"/>
+      <c r="N37" s="123"/>
+      <c r="O37" s="123"/>
+      <c r="P37" s="123"/>
+      <c r="Q37" s="123"/>
+      <c r="R37" s="123"/>
+      <c r="S37" s="123"/>
+      <c r="T37" s="123"/>
       <c r="U37" s="114"/>
     </row>
-    <row r="38" ht="19.5" customHeight="1">
-      <c r="A38" s="124" t="s">
-        <v>54</v>
-      </c>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="26"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="27"/>
       <c r="D38" s="27"/>
       <c r="E38" s="27"/>
-      <c r="F38" s="125" t="s">
-        <v>55</v>
-      </c>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27"/>
       <c r="J38" s="27"/>
-      <c r="K38" s="125" t="s">
-        <v>56</v>
-      </c>
+      <c r="K38" s="27"/>
+      <c r="L38" s="27"/>
+      <c r="M38" s="27"/>
       <c r="N38" s="27"/>
       <c r="O38" s="27"/>
-      <c r="P38" s="125" t="s">
-        <v>57</v>
-      </c>
+      <c r="P38" s="27"/>
       <c r="Q38" s="27"/>
-      <c r="R38" s="125" t="s">
-        <v>58</v>
-      </c>
-      <c r="U38" s="11"/>
+      <c r="R38" s="27"/>
+      <c r="S38" s="27"/>
+      <c r="T38" s="27"/>
+      <c r="U38" s="114"/>
     </row>
     <row r="39" ht="19.5" customHeight="1">
-      <c r="A39" s="10"/>
+      <c r="A39" s="124" t="s">
+        <v>56</v>
+      </c>
       <c r="D39" s="27"/>
       <c r="E39" s="27"/>
+      <c r="F39" s="125" t="s">
+        <v>57</v>
+      </c>
       <c r="J39" s="27"/>
+      <c r="K39" s="125" t="s">
+        <v>58</v>
+      </c>
       <c r="N39" s="27"/>
       <c r="O39" s="27"/>
+      <c r="P39" s="125" t="s">
+        <v>59</v>
+      </c>
       <c r="Q39" s="27"/>
+      <c r="R39" s="125" t="s">
+        <v>60</v>
+      </c>
       <c r="U39" s="11"/>
     </row>
     <row r="40" ht="19.5" customHeight="1">
-      <c r="A40" s="126"/>
-      <c r="B40" s="120"/>
-      <c r="C40" s="120"/>
-      <c r="D40" s="127"/>
-      <c r="E40" s="127"/>
-      <c r="F40" s="120"/>
-      <c r="G40" s="120"/>
-      <c r="H40" s="120"/>
-      <c r="I40" s="120"/>
-      <c r="J40" s="127"/>
-      <c r="K40" s="120"/>
-      <c r="L40" s="120"/>
-      <c r="M40" s="120"/>
-      <c r="N40" s="127"/>
-      <c r="O40" s="127"/>
-      <c r="P40" s="120"/>
-      <c r="Q40" s="127"/>
-      <c r="R40" s="120"/>
-      <c r="S40" s="120"/>
-      <c r="T40" s="120"/>
-      <c r="U40" s="42"/>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="128"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1"/>
+      <c r="A40" s="10"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="N40" s="27"/>
+      <c r="O40" s="27"/>
+      <c r="Q40" s="27"/>
+      <c r="U40" s="11"/>
+    </row>
+    <row r="41" ht="19.5" customHeight="1">
+      <c r="A41" s="126"/>
+      <c r="B41" s="120"/>
+      <c r="C41" s="120"/>
+      <c r="D41" s="127"/>
+      <c r="E41" s="127"/>
+      <c r="F41" s="120"/>
+      <c r="G41" s="120"/>
+      <c r="H41" s="120"/>
+      <c r="I41" s="120"/>
+      <c r="J41" s="127"/>
+      <c r="K41" s="120"/>
+      <c r="L41" s="120"/>
+      <c r="M41" s="120"/>
+      <c r="N41" s="127"/>
+      <c r="O41" s="127"/>
+      <c r="P41" s="120"/>
+      <c r="Q41" s="127"/>
+      <c r="R41" s="120"/>
+      <c r="S41" s="120"/>
+      <c r="T41" s="120"/>
+      <c r="U41" s="42"/>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="128"/>
+    </row>
     <row r="43" ht="15.75" customHeight="1"/>
     <row r="44" ht="15.75" customHeight="1"/>
     <row r="45" ht="15.75" customHeight="1"/>
@@ -3581,29 +3612,33 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="43">
     <mergeCell ref="O10:P10"/>
-    <mergeCell ref="Q13:T13"/>
-    <mergeCell ref="K27:M27"/>
-    <mergeCell ref="R27:T27"/>
+    <mergeCell ref="Q14:T14"/>
+    <mergeCell ref="O11:P11"/>
     <mergeCell ref="K28:M28"/>
     <mergeCell ref="R28:T28"/>
-    <mergeCell ref="H32:T33"/>
-    <mergeCell ref="C35:T35"/>
-    <mergeCell ref="A38:C40"/>
-    <mergeCell ref="F38:I40"/>
-    <mergeCell ref="K38:M40"/>
-    <mergeCell ref="P38:P40"/>
-    <mergeCell ref="R38:U40"/>
-    <mergeCell ref="A41:U42"/>
+    <mergeCell ref="K29:M29"/>
+    <mergeCell ref="R29:T29"/>
+    <mergeCell ref="H33:T34"/>
+    <mergeCell ref="C36:T36"/>
+    <mergeCell ref="A39:C41"/>
+    <mergeCell ref="F39:I41"/>
+    <mergeCell ref="K39:M41"/>
+    <mergeCell ref="P39:P41"/>
+    <mergeCell ref="R39:U41"/>
+    <mergeCell ref="A42:U43"/>
+    <mergeCell ref="K26:M26"/>
+    <mergeCell ref="K27:M27"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="G5:M5"/>
     <mergeCell ref="N5:Q5"/>
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="T6:U6"/>
-    <mergeCell ref="A7:F33"/>
     <mergeCell ref="J7:M7"/>
+    <mergeCell ref="A7:F34"/>
     <mergeCell ref="A1:A4"/>
     <mergeCell ref="B1:D4"/>
     <mergeCell ref="E1:P4"/>
@@ -3615,14 +3650,14 @@
     <mergeCell ref="O7:P7"/>
     <mergeCell ref="O8:P8"/>
     <mergeCell ref="O9:P9"/>
-    <mergeCell ref="R15:T15"/>
     <mergeCell ref="R16:T16"/>
     <mergeCell ref="R17:T17"/>
     <mergeCell ref="R18:T18"/>
-    <mergeCell ref="J23:M23"/>
-    <mergeCell ref="Q23:T23"/>
-    <mergeCell ref="R25:T25"/>
+    <mergeCell ref="R19:T19"/>
+    <mergeCell ref="J24:M24"/>
+    <mergeCell ref="Q24:T24"/>
     <mergeCell ref="R26:T26"/>
+    <mergeCell ref="R27:T27"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins bottom="0.0" footer="0.0" header="0.0" left="0.0" right="0.0" top="0.393700787401575"/>

</xml_diff>

<commit_message>
fix: update IATF export template formatting
</commit_message>
<xml_diff>
--- a/sheet_cutting_layout/templates/iatf/sheet_cutting_layout.xlsx
+++ b/sheet_cutting_layout/templates/iatf/sheet_cutting_layout.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="60">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -34,27 +34,21 @@
     <t>Sheet Cutting Layout No:-</t>
   </si>
   <si>
-    <t>Part Name:PANO BRKT ASSY GRIP MTG FRT LH</t>
-  </si>
-  <si>
-    <t>Part Number:-0101ES205450N</t>
+    <t>Part Name:</t>
+  </si>
+  <si>
+    <t>Part Number:</t>
   </si>
   <si>
     <t xml:space="preserve">Project </t>
   </si>
   <si>
-    <t>S225</t>
-  </si>
-  <si>
     <t>Wt /sheet</t>
   </si>
   <si>
     <t>Raw Material Grade</t>
   </si>
   <si>
-    <t>HSLA-340</t>
-  </si>
-  <si>
     <t>BOM</t>
   </si>
   <si>
@@ -140,6 +134,9 @@
   </si>
   <si>
     <t xml:space="preserve">Scrap Weight of a Part:-                           </t>
+  </si>
+  <si>
+    <t>Kg</t>
   </si>
   <si>
     <t>I</t>
@@ -803,7 +800,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="130">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -843,9 +840,12 @@
     <xf borderId="19" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="20" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="21" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="22" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="18" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="19" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -854,9 +854,6 @@
     </xf>
     <xf borderId="23" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1006,7 +1003,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="35" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="11" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
@@ -1019,6 +1016,9 @@
     </xf>
     <xf borderId="38" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="38" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="38" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1474,38 +1474,32 @@
       <c r="K5" s="20"/>
       <c r="L5" s="20"/>
       <c r="M5" s="23"/>
-      <c r="N5" s="19" t="s">
+      <c r="N5" s="24" t="s">
         <v>8</v>
       </c>
       <c r="O5" s="20"/>
       <c r="P5" s="20"/>
       <c r="Q5" s="20"/>
-      <c r="R5" s="24"/>
-      <c r="S5" s="24"/>
-      <c r="T5" s="24"/>
-      <c r="U5" s="25"/>
+      <c r="R5" s="25"/>
+      <c r="S5" s="25"/>
+      <c r="T5" s="25"/>
+      <c r="U5" s="26"/>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="28"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="28"/>
+      <c r="M6" s="28"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="30" t="s">
         <v>10</v>
-      </c>
-      <c r="C6" s="28"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-      <c r="O6" s="30" t="s">
-        <v>11</v>
       </c>
       <c r="P6" s="31"/>
       <c r="Q6" s="32">
@@ -1535,33 +1529,31 @@
         <v>1.0</v>
       </c>
       <c r="I7" s="38" t="s">
-        <v>12</v>
-      </c>
-      <c r="J7" s="39" t="s">
-        <v>13</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J7" s="39"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
       <c r="M7" s="8"/>
       <c r="N7" s="40"/>
       <c r="O7" s="41" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="P7" s="42"/>
       <c r="Q7" s="43" t="s">
+        <v>13</v>
+      </c>
+      <c r="R7" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="S7" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="R7" s="43" t="s">
+      <c r="T7" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="S7" s="43" t="s">
+      <c r="U7" s="44" t="s">
         <v>17</v>
-      </c>
-      <c r="T7" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="U7" s="44" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -1572,40 +1564,38 @@
         <v>2.0</v>
       </c>
       <c r="I8" s="47" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J8" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="K8" s="49">
-        <v>1.6</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K8" s="49"/>
       <c r="L8" s="48"/>
       <c r="M8" s="50"/>
       <c r="N8" s="40"/>
       <c r="O8" s="51" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="P8" s="52"/>
-      <c r="Q8" s="53">
+      <c r="Q8" s="53" t="str">
         <f>+K15</f>
-        <v>0.73622</v>
-      </c>
-      <c r="R8" s="53">
+        <v/>
+      </c>
+      <c r="R8" s="53" t="str">
         <f>+K16</f>
-        <v>0.292</v>
-      </c>
-      <c r="S8" s="54">
+        <v/>
+      </c>
+      <c r="S8" s="54" t="str">
         <f>+K17</f>
-        <v>0.44422</v>
-      </c>
-      <c r="T8" s="55">
+        <v/>
+      </c>
+      <c r="T8" s="55" t="str">
         <f>+K14</f>
-        <v>48</v>
+        <v/>
       </c>
       <c r="U8" s="56">
         <f>+T8*Q8</f>
-        <v>35.33856</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1616,42 +1606,32 @@
         <v>3.0</v>
       </c>
       <c r="I9" s="47" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J9" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="K9" s="49">
-        <v>1.6</v>
-      </c>
-      <c r="L9" s="48">
-        <v>1250.0</v>
-      </c>
-      <c r="M9" s="50">
-        <v>2500.0</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K9" s="49"/>
+      <c r="L9" s="48"/>
+      <c r="M9" s="50"/>
       <c r="N9" s="40"/>
       <c r="O9" s="57" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="P9" s="52"/>
-      <c r="Q9" s="53">
+      <c r="Q9" s="53" t="str">
         <f>+K28</f>
-        <v>3.96144</v>
-      </c>
-      <c r="R9" s="53">
-        <v>0.0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="R9" s="53"/>
       <c r="S9" s="58" t="str">
         <f>K29</f>
         <v/>
       </c>
-      <c r="T9" s="55">
-        <v>1.0</v>
-      </c>
+      <c r="T9" s="55"/>
       <c r="U9" s="56">
         <f>+Q9*T9</f>
-        <v>3.96144</v>
+        <v>0</v>
       </c>
       <c r="W9" s="59"/>
     </row>
@@ -1663,39 +1643,31 @@
         <v>4.0</v>
       </c>
       <c r="I10" s="47" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J10" s="48" t="s">
-        <v>26</v>
-      </c>
-      <c r="K10" s="60">
-        <f>+K11*L11*M11*0.786/100000</f>
-        <v>4.41732</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="K10" s="60"/>
       <c r="L10" s="49"/>
       <c r="M10" s="61"/>
       <c r="N10" s="40"/>
       <c r="O10" s="57" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="P10" s="52"/>
-      <c r="Q10" s="53">
-        <f t="shared" ref="Q10:Q11" si="1">R17+R27</f>
-        <v>0</v>
-      </c>
+      <c r="Q10" s="53"/>
       <c r="R10" s="53" t="str">
-        <f t="shared" ref="R10:R11" si="2">R18</f>
+        <f t="shared" ref="R10:R11" si="1">R18</f>
         <v/>
       </c>
       <c r="S10" s="53" t="str">
-        <f t="shared" ref="S10:S11" si="3">R19</f>
+        <f t="shared" ref="S10:S11" si="2">R19</f>
         <v/>
       </c>
-      <c r="T10" s="55">
-        <v>1.0</v>
-      </c>
+      <c r="T10" s="55"/>
       <c r="U10" s="56">
-        <f t="shared" ref="U10:U11" si="4">T10*Q10</f>
+        <f t="shared" ref="U10:U11" si="3">T10*Q10</f>
         <v>0</v>
       </c>
     </row>
@@ -1707,42 +1679,31 @@
         <v>5.0</v>
       </c>
       <c r="I11" s="47" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J11" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="K11" s="48">
-        <v>1.6</v>
-      </c>
-      <c r="L11" s="48">
-        <v>1250.0</v>
-      </c>
-      <c r="M11" s="50">
-        <v>281.0</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="K11" s="48"/>
+      <c r="L11" s="48"/>
+      <c r="M11" s="50"/>
       <c r="N11" s="40"/>
       <c r="O11" s="62" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="P11" s="63"/>
-      <c r="Q11" s="64">
+      <c r="Q11" s="64"/>
+      <c r="R11" s="64" t="str">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R11" s="64" t="str">
+        <v/>
+      </c>
+      <c r="S11" s="64" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="S11" s="64" t="str">
+      <c r="T11" s="65"/>
+      <c r="U11" s="66">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="T11" s="65">
-        <v>1.0</v>
-      </c>
-      <c r="U11" s="66">
-        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -1754,14 +1715,12 @@
         <v>6.0</v>
       </c>
       <c r="I12" s="47" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J12" s="48" t="s">
-        <v>31</v>
-      </c>
-      <c r="K12" s="67">
-        <v>6.0</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="K12" s="67"/>
       <c r="L12" s="48"/>
       <c r="M12" s="50"/>
       <c r="N12" s="40"/>
@@ -1773,7 +1732,7 @@
       <c r="T12" s="40"/>
       <c r="U12" s="69">
         <f>SUM(U8:U11)</f>
-        <v>39.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1784,36 +1743,34 @@
         <v>7.0</v>
       </c>
       <c r="I13" s="47" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J13" s="48" t="s">
-        <v>31</v>
-      </c>
-      <c r="K13" s="67">
-        <v>8.0</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="K13" s="67"/>
       <c r="L13" s="48"/>
       <c r="M13" s="50"/>
       <c r="N13" s="40"/>
       <c r="O13" s="70" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="P13" s="71" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="Q13" s="72" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R13" s="73" t="str">
-        <f t="shared" ref="R13:T13" si="5">K19</f>
+        <f t="shared" ref="R13:T13" si="4">K19</f>
         <v/>
       </c>
       <c r="S13" s="73" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="T13" s="74" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="U13" s="75"/>
@@ -1826,15 +1783,12 @@
         <v>8.0</v>
       </c>
       <c r="I14" s="47" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J14" s="48" t="s">
-        <v>31</v>
-      </c>
-      <c r="K14" s="48">
-        <f>+K13*K12</f>
-        <v>48</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="K14" s="48"/>
       <c r="L14" s="48"/>
       <c r="M14" s="50"/>
       <c r="N14" s="40"/>
@@ -1842,7 +1796,7 @@
         <v>1.0</v>
       </c>
       <c r="P14" s="76" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Q14" s="77"/>
       <c r="R14" s="13"/>
@@ -1860,15 +1814,12 @@
         <v>9.0</v>
       </c>
       <c r="I15" s="47" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J15" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="K15" s="81">
-        <f>+(K10/K12)</f>
-        <v>0.73622</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="K15" s="81"/>
       <c r="L15" s="60"/>
       <c r="M15" s="82"/>
       <c r="N15" s="40"/>
@@ -1876,26 +1827,26 @@
         <v>2.0</v>
       </c>
       <c r="P15" s="76" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="Q15" s="48" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R15" s="83" t="str">
-        <f t="shared" ref="R15:T15" si="6">R13</f>
+        <f t="shared" ref="R15:T15" si="5">R13</f>
         <v/>
       </c>
       <c r="S15" s="83" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="T15" s="50" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="U15" s="75"/>
-      <c r="W15" s="27"/>
-      <c r="X15" s="27"/>
+      <c r="W15" s="28"/>
+      <c r="X15" s="28"/>
     </row>
     <row r="16">
       <c r="A16" s="45"/>
@@ -1905,14 +1856,12 @@
         <v>10.0</v>
       </c>
       <c r="I16" s="47" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J16" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="K16" s="81">
-        <v>0.292</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="K16" s="81"/>
       <c r="L16" s="48"/>
       <c r="M16" s="50"/>
       <c r="N16" s="40"/>
@@ -1920,17 +1869,17 @@
         <v>3.0</v>
       </c>
       <c r="P16" s="76" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="Q16" s="48" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="R16" s="83"/>
       <c r="S16" s="13"/>
       <c r="T16" s="14"/>
       <c r="U16" s="75"/>
       <c r="W16" s="84"/>
-      <c r="X16" s="27"/>
+      <c r="X16" s="28"/>
     </row>
     <row r="17">
       <c r="A17" s="45"/>
@@ -1940,15 +1889,12 @@
         <v>11.0</v>
       </c>
       <c r="I17" s="47" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J17" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="K17" s="60">
-        <f>+K15-K16</f>
-        <v>0.44422</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="K17" s="60"/>
       <c r="L17" s="60"/>
       <c r="M17" s="82"/>
       <c r="N17" s="40"/>
@@ -1956,10 +1902,10 @@
         <v>4.0</v>
       </c>
       <c r="P17" s="76" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q17" s="85" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="R17" s="86">
         <f>+R15*S15*T15*0.786/100000</f>
@@ -1968,138 +1914,134 @@
       <c r="S17" s="13"/>
       <c r="T17" s="14"/>
       <c r="U17" s="75"/>
-      <c r="W17" s="27"/>
-      <c r="X17" s="27"/>
+      <c r="W17" s="28"/>
+      <c r="X17" s="28"/>
     </row>
     <row r="18">
       <c r="A18" s="45"/>
       <c r="F18" s="11"/>
       <c r="G18" s="29"/>
       <c r="H18" s="87" t="s">
+        <v>42</v>
+      </c>
+      <c r="I18" s="88" t="s">
         <v>43</v>
       </c>
-      <c r="I18" s="88" t="s">
-        <v>44</v>
-      </c>
       <c r="J18" s="89" t="s">
-        <v>21</v>
-      </c>
-      <c r="K18" s="49">
+        <v>19</v>
+      </c>
+      <c r="K18" s="49" t="str">
         <f>+K8</f>
-        <v>1.6</v>
-      </c>
-      <c r="L18" s="48">
-        <v>252.0</v>
-      </c>
-      <c r="M18" s="50">
-        <v>1250.0</v>
-      </c>
+        <v/>
+      </c>
+      <c r="L18" s="48"/>
+      <c r="M18" s="50"/>
       <c r="N18" s="40"/>
       <c r="O18" s="46">
         <v>5.0</v>
       </c>
       <c r="P18" s="76" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q18" s="48" t="s">
         <v>38</v>
+      </c>
+      <c r="Q18" s="90" t="s">
+        <v>41</v>
       </c>
       <c r="R18" s="86"/>
       <c r="S18" s="13"/>
       <c r="T18" s="14"/>
       <c r="U18" s="75"/>
-      <c r="V18" s="90" t="s">
+      <c r="V18" s="91" t="s">
         <v>0</v>
       </c>
-      <c r="W18" s="27"/>
-      <c r="X18" s="27"/>
+      <c r="W18" s="28"/>
+      <c r="X18" s="28"/>
     </row>
     <row r="19">
       <c r="A19" s="45"/>
       <c r="F19" s="11"/>
       <c r="G19" s="29"/>
       <c r="H19" s="87" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I19" s="88" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J19" s="89" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K19" s="48"/>
-      <c r="L19" s="91"/>
+      <c r="L19" s="92"/>
       <c r="M19" s="50"/>
       <c r="N19" s="40"/>
       <c r="O19" s="46">
         <v>6.0</v>
       </c>
       <c r="P19" s="76" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q19" s="48" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="Q19" s="90" t="s">
+        <v>41</v>
       </c>
       <c r="R19" s="86"/>
       <c r="S19" s="13"/>
       <c r="T19" s="14"/>
       <c r="U19" s="75"/>
-      <c r="W19" s="27"/>
-      <c r="X19" s="27"/>
+      <c r="W19" s="28"/>
+      <c r="X19" s="28"/>
     </row>
     <row r="20">
       <c r="A20" s="45"/>
       <c r="F20" s="11"/>
       <c r="G20" s="29"/>
-      <c r="H20" s="92" t="s">
+      <c r="H20" s="93" t="s">
+        <v>44</v>
+      </c>
+      <c r="I20" s="94" t="s">
         <v>45</v>
       </c>
-      <c r="I20" s="93" t="s">
-        <v>46</v>
-      </c>
-      <c r="J20" s="94" t="s">
-        <v>21</v>
-      </c>
-      <c r="K20" s="95"/>
-      <c r="L20" s="95"/>
-      <c r="M20" s="96"/>
+      <c r="J20" s="95" t="s">
+        <v>19</v>
+      </c>
+      <c r="K20" s="96"/>
+      <c r="L20" s="96"/>
+      <c r="M20" s="97"/>
       <c r="N20" s="40"/>
       <c r="O20" s="46">
         <v>7.0</v>
       </c>
-      <c r="P20" s="97" t="s">
-        <v>47</v>
+      <c r="P20" s="98" t="s">
+        <v>46</v>
       </c>
       <c r="Q20" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="R20" s="98"/>
-      <c r="S20" s="98"/>
-      <c r="T20" s="99"/>
+        <v>19</v>
+      </c>
+      <c r="R20" s="99"/>
+      <c r="S20" s="99"/>
+      <c r="T20" s="100"/>
       <c r="U20" s="75"/>
-      <c r="W20" s="27"/>
-      <c r="X20" s="27"/>
+      <c r="W20" s="28"/>
+      <c r="X20" s="28"/>
     </row>
     <row r="21">
       <c r="A21" s="45"/>
       <c r="F21" s="11"/>
       <c r="G21" s="29"/>
       <c r="N21" s="40"/>
-      <c r="O21" s="100">
+      <c r="O21" s="101">
         <v>8.0</v>
       </c>
-      <c r="P21" s="101" t="s">
-        <v>48</v>
+      <c r="P21" s="102" t="s">
+        <v>47</v>
       </c>
       <c r="Q21" s="65" t="s">
-        <v>21</v>
-      </c>
-      <c r="R21" s="102"/>
-      <c r="S21" s="102"/>
-      <c r="T21" s="103"/>
+        <v>19</v>
+      </c>
+      <c r="R21" s="103"/>
+      <c r="S21" s="103"/>
+      <c r="T21" s="104"/>
       <c r="U21" s="75"/>
-      <c r="W21" s="27"/>
-      <c r="X21" s="27"/>
+      <c r="W21" s="28"/>
+      <c r="X21" s="28"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="45"/>
@@ -2112,66 +2054,66 @@
       <c r="L22" s="40"/>
       <c r="M22" s="40"/>
       <c r="N22" s="40"/>
-      <c r="O22" s="27"/>
-      <c r="P22" s="27"/>
-      <c r="Q22" s="27"/>
-      <c r="R22" s="27"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
+      <c r="O22" s="28"/>
+      <c r="P22" s="28"/>
+      <c r="Q22" s="28"/>
+      <c r="R22" s="28"/>
+      <c r="S22" s="28"/>
+      <c r="T22" s="28"/>
       <c r="U22" s="75"/>
-      <c r="W22" s="27"/>
-      <c r="X22" s="27"/>
+      <c r="W22" s="28"/>
+      <c r="X22" s="28"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="45"/>
       <c r="F23" s="11"/>
       <c r="G23" s="29"/>
-      <c r="H23" s="104" t="s">
-        <v>43</v>
-      </c>
-      <c r="I23" s="105" t="s">
-        <v>49</v>
+      <c r="H23" s="105" t="s">
+        <v>42</v>
+      </c>
+      <c r="I23" s="106" t="s">
+        <v>48</v>
       </c>
       <c r="J23" s="72" t="s">
-        <v>21</v>
-      </c>
-      <c r="K23" s="106">
-        <f t="shared" ref="K23:M23" si="7">+K18</f>
-        <v>1.6</v>
-      </c>
-      <c r="L23" s="72">
+        <v>19</v>
+      </c>
+      <c r="K23" s="107" t="str">
+        <f t="shared" ref="K23:M23" si="6">+K18</f>
+        <v/>
+      </c>
+      <c r="L23" s="72" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="M23" s="108" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="N23" s="40"/>
+      <c r="O23" s="105" t="s">
+        <v>44</v>
+      </c>
+      <c r="P23" s="109" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q23" s="72" t="s">
+        <v>19</v>
+      </c>
+      <c r="R23" s="72" t="str">
+        <f t="shared" ref="R23:T23" si="7">K20</f>
+        <v/>
+      </c>
+      <c r="S23" s="72" t="str">
         <f t="shared" si="7"/>
-        <v>252</v>
-      </c>
-      <c r="M23" s="107">
+        <v/>
+      </c>
+      <c r="T23" s="72" t="str">
         <f t="shared" si="7"/>
-        <v>1250</v>
-      </c>
-      <c r="N23" s="40"/>
-      <c r="O23" s="104" t="s">
-        <v>45</v>
-      </c>
-      <c r="P23" s="108" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q23" s="72" t="s">
-        <v>21</v>
-      </c>
-      <c r="R23" s="72" t="str">
-        <f t="shared" ref="R23:T23" si="8">K20</f>
         <v/>
       </c>
-      <c r="S23" s="72" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="T23" s="72" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
       <c r="U23" s="75"/>
-      <c r="W23" s="109"/>
-      <c r="X23" s="27"/>
+      <c r="W23" s="110"/>
+      <c r="X23" s="28"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="45"/>
@@ -2181,7 +2123,7 @@
         <v>1.0</v>
       </c>
       <c r="I24" s="47" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J24" s="83"/>
       <c r="K24" s="13"/>
@@ -2192,15 +2134,15 @@
         <v>1.0</v>
       </c>
       <c r="P24" s="76" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Q24" s="83"/>
       <c r="R24" s="13"/>
       <c r="S24" s="13"/>
       <c r="T24" s="14"/>
       <c r="U24" s="75"/>
-      <c r="W24" s="27"/>
-      <c r="X24" s="27"/>
+      <c r="W24" s="28"/>
+      <c r="X24" s="28"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="45"/>
@@ -2210,48 +2152,48 @@
         <v>2.0</v>
       </c>
       <c r="I25" s="47" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J25" s="48" t="s">
-        <v>21</v>
-      </c>
-      <c r="K25" s="49">
-        <f t="shared" ref="K25:M25" si="9">+K23</f>
-        <v>1.6</v>
-      </c>
-      <c r="L25" s="48">
-        <f t="shared" si="9"/>
-        <v>252</v>
-      </c>
-      <c r="M25" s="50">
-        <f t="shared" si="9"/>
-        <v>1250</v>
+        <v>19</v>
+      </c>
+      <c r="K25" s="49" t="str">
+        <f t="shared" ref="K25:M25" si="8">+K23</f>
+        <v/>
+      </c>
+      <c r="L25" s="48" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="M25" s="50" t="str">
+        <f t="shared" si="8"/>
+        <v/>
       </c>
       <c r="N25" s="40"/>
       <c r="O25" s="46">
         <v>2.0</v>
       </c>
       <c r="P25" s="76" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="Q25" s="48" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R25" s="83" t="str">
-        <f t="shared" ref="R25:T25" si="10">+R23</f>
+        <f t="shared" ref="R25:T25" si="9">+R23</f>
         <v/>
       </c>
       <c r="S25" s="83" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="T25" s="110" t="str">
-        <f t="shared" si="10"/>
+      <c r="T25" s="111" t="str">
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="U25" s="75"/>
-      <c r="W25" s="27"/>
-      <c r="X25" s="27"/>
+      <c r="W25" s="28"/>
+      <c r="X25" s="28"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="45"/>
@@ -2261,10 +2203,10 @@
         <v>3.0</v>
       </c>
       <c r="I26" s="47" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J26" s="48" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K26" s="83"/>
       <c r="L26" s="13"/>
@@ -2274,17 +2216,17 @@
         <v>3.0</v>
       </c>
       <c r="P26" s="76" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="Q26" s="48" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="R26" s="83"/>
       <c r="S26" s="13"/>
       <c r="T26" s="14"/>
       <c r="U26" s="75"/>
-      <c r="W26" s="27"/>
-      <c r="X26" s="27"/>
+      <c r="W26" s="28"/>
+      <c r="X26" s="28"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="45"/>
@@ -2294,10 +2236,10 @@
         <v>4.0</v>
       </c>
       <c r="I27" s="47" t="s">
-        <v>37</v>
-      </c>
-      <c r="J27" s="48" t="s">
-        <v>31</v>
+        <v>35</v>
+      </c>
+      <c r="J27" s="90" t="s">
+        <v>41</v>
       </c>
       <c r="K27" s="86"/>
       <c r="L27" s="13"/>
@@ -2307,10 +2249,10 @@
         <v>4.0</v>
       </c>
       <c r="P27" s="76" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q27" s="48" t="s">
-        <v>38</v>
+        <v>35</v>
+      </c>
+      <c r="Q27" s="90" t="s">
+        <v>41</v>
       </c>
       <c r="R27" s="86">
         <f>+R25*S25*T25*0.786/100000</f>
@@ -2319,8 +2261,8 @@
       <c r="S27" s="13"/>
       <c r="T27" s="14"/>
       <c r="U27" s="75"/>
-      <c r="W27" s="27"/>
-      <c r="X27" s="27"/>
+      <c r="W27" s="28"/>
+      <c r="X27" s="28"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="45"/>
@@ -2330,15 +2272,12 @@
         <v>5.0</v>
       </c>
       <c r="I28" s="47" t="s">
-        <v>40</v>
-      </c>
-      <c r="J28" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="K28" s="86">
-        <f>+K25*L25*M25*0.786/100000</f>
-        <v>3.96144</v>
-      </c>
+      <c r="J28" s="90" t="s">
+        <v>41</v>
+      </c>
+      <c r="K28" s="86"/>
       <c r="L28" s="13"/>
       <c r="M28" s="14"/>
       <c r="N28" s="40"/>
@@ -2346,18 +2285,18 @@
         <v>5.0</v>
       </c>
       <c r="P28" s="76" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q28" s="48" t="s">
         <v>38</v>
+      </c>
+      <c r="Q28" s="90" t="s">
+        <v>41</v>
       </c>
       <c r="R28" s="83"/>
       <c r="S28" s="13"/>
       <c r="T28" s="14"/>
       <c r="U28" s="75"/>
-      <c r="W28" s="27"/>
-      <c r="X28" s="27"/>
-      <c r="Z28" s="111"/>
+      <c r="W28" s="28"/>
+      <c r="X28" s="28"/>
+      <c r="Z28" s="112"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="45"/>
@@ -2367,10 +2306,10 @@
         <v>6.0</v>
       </c>
       <c r="I29" s="47" t="s">
-        <v>42</v>
-      </c>
-      <c r="J29" s="48" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="J29" s="90" t="s">
+        <v>41</v>
       </c>
       <c r="K29" s="86"/>
       <c r="L29" s="13"/>
@@ -2380,17 +2319,17 @@
         <v>6.0</v>
       </c>
       <c r="P29" s="76" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q29" s="48" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="Q29" s="90" t="s">
+        <v>41</v>
       </c>
       <c r="R29" s="83"/>
       <c r="S29" s="13"/>
       <c r="T29" s="14"/>
       <c r="U29" s="75"/>
-      <c r="W29" s="27"/>
-      <c r="X29" s="27"/>
+      <c r="W29" s="28"/>
+      <c r="X29" s="28"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="45"/>
@@ -2399,86 +2338,86 @@
       <c r="H30" s="46">
         <v>7.0</v>
       </c>
-      <c r="I30" s="112" t="s">
-        <v>50</v>
+      <c r="I30" s="113" t="s">
+        <v>49</v>
       </c>
       <c r="J30" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="K30" s="98"/>
-      <c r="L30" s="98"/>
-      <c r="M30" s="99"/>
-      <c r="N30" s="113"/>
+        <v>19</v>
+      </c>
+      <c r="K30" s="99"/>
+      <c r="L30" s="99"/>
+      <c r="M30" s="100"/>
+      <c r="N30" s="114"/>
       <c r="O30" s="46">
         <v>7.0</v>
       </c>
-      <c r="P30" s="97" t="s">
-        <v>51</v>
+      <c r="P30" s="98" t="s">
+        <v>50</v>
       </c>
       <c r="Q30" s="55" t="s">
-        <v>21</v>
-      </c>
-      <c r="R30" s="98"/>
-      <c r="S30" s="98"/>
-      <c r="T30" s="99"/>
-      <c r="U30" s="114"/>
+        <v>19</v>
+      </c>
+      <c r="R30" s="99"/>
+      <c r="S30" s="99"/>
+      <c r="T30" s="100"/>
+      <c r="U30" s="115"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="45"/>
       <c r="F31" s="11"/>
       <c r="G31" s="29"/>
-      <c r="H31" s="100">
+      <c r="H31" s="101">
         <v>8.0</v>
       </c>
-      <c r="I31" s="115" t="s">
+      <c r="I31" s="116" t="s">
+        <v>51</v>
+      </c>
+      <c r="J31" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="K31" s="103"/>
+      <c r="L31" s="103"/>
+      <c r="M31" s="104"/>
+      <c r="N31" s="114"/>
+      <c r="O31" s="101">
+        <v>8.0</v>
+      </c>
+      <c r="P31" s="102" t="s">
         <v>52</v>
       </c>
-      <c r="J31" s="65" t="s">
-        <v>21</v>
-      </c>
-      <c r="K31" s="102"/>
-      <c r="L31" s="102"/>
-      <c r="M31" s="103"/>
-      <c r="N31" s="113"/>
-      <c r="O31" s="100">
-        <v>8.0</v>
-      </c>
-      <c r="P31" s="101" t="s">
-        <v>53</v>
-      </c>
       <c r="Q31" s="65" t="s">
-        <v>21</v>
-      </c>
-      <c r="R31" s="102"/>
-      <c r="S31" s="102"/>
-      <c r="T31" s="103"/>
-      <c r="U31" s="114"/>
+        <v>19</v>
+      </c>
+      <c r="R31" s="103"/>
+      <c r="S31" s="103"/>
+      <c r="T31" s="104"/>
+      <c r="U31" s="115"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="45"/>
       <c r="F32" s="11"/>
       <c r="G32" s="29"/>
       <c r="H32" s="68"/>
-      <c r="I32" s="116"/>
-      <c r="J32" s="116"/>
-      <c r="K32" s="116"/>
-      <c r="L32" s="116"/>
-      <c r="M32" s="116"/>
-      <c r="N32" s="116"/>
-      <c r="O32" s="116"/>
-      <c r="P32" s="116"/>
-      <c r="Q32" s="27"/>
-      <c r="R32" s="27"/>
-      <c r="S32" s="27"/>
-      <c r="T32" s="27"/>
-      <c r="U32" s="114"/>
+      <c r="I32" s="117"/>
+      <c r="J32" s="117"/>
+      <c r="K32" s="117"/>
+      <c r="L32" s="117"/>
+      <c r="M32" s="117"/>
+      <c r="N32" s="117"/>
+      <c r="O32" s="117"/>
+      <c r="P32" s="117"/>
+      <c r="Q32" s="28"/>
+      <c r="R32" s="28"/>
+      <c r="S32" s="28"/>
+      <c r="T32" s="28"/>
+      <c r="U32" s="115"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="45"/>
       <c r="F33" s="11"/>
       <c r="G33" s="29"/>
-      <c r="H33" s="117" t="s">
-        <v>54</v>
+      <c r="H33" s="118" t="s">
+        <v>53</v>
       </c>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
@@ -2491,168 +2430,168 @@
       <c r="Q33" s="3"/>
       <c r="R33" s="3"/>
       <c r="S33" s="3"/>
-      <c r="T33" s="118"/>
-      <c r="U33" s="114"/>
+      <c r="T33" s="119"/>
+      <c r="U33" s="115"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="119"/>
-      <c r="B34" s="120"/>
-      <c r="C34" s="120"/>
-      <c r="D34" s="120"/>
-      <c r="E34" s="120"/>
+      <c r="A34" s="120"/>
+      <c r="B34" s="121"/>
+      <c r="C34" s="121"/>
+      <c r="D34" s="121"/>
+      <c r="E34" s="121"/>
       <c r="F34" s="42"/>
       <c r="G34" s="29"/>
-      <c r="H34" s="121"/>
-      <c r="I34" s="122"/>
-      <c r="J34" s="122"/>
-      <c r="K34" s="122"/>
-      <c r="L34" s="122"/>
-      <c r="M34" s="122"/>
-      <c r="N34" s="122"/>
-      <c r="O34" s="122"/>
-      <c r="P34" s="122"/>
-      <c r="Q34" s="122"/>
-      <c r="R34" s="122"/>
-      <c r="S34" s="122"/>
+      <c r="H34" s="122"/>
+      <c r="I34" s="123"/>
+      <c r="J34" s="123"/>
+      <c r="K34" s="123"/>
+      <c r="L34" s="123"/>
+      <c r="M34" s="123"/>
+      <c r="N34" s="123"/>
+      <c r="O34" s="123"/>
+      <c r="P34" s="123"/>
+      <c r="Q34" s="123"/>
+      <c r="R34" s="123"/>
+      <c r="S34" s="123"/>
       <c r="T34" s="34"/>
-      <c r="U34" s="114"/>
+      <c r="U34" s="115"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="26"/>
-      <c r="B35" s="27"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
+      <c r="A35" s="27"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
       <c r="G35" s="29"/>
-      <c r="H35" s="123"/>
-      <c r="I35" s="123"/>
-      <c r="J35" s="123"/>
-      <c r="K35" s="123"/>
-      <c r="L35" s="123"/>
-      <c r="M35" s="123"/>
-      <c r="N35" s="123"/>
-      <c r="O35" s="123"/>
-      <c r="P35" s="123"/>
-      <c r="Q35" s="123"/>
-      <c r="R35" s="123"/>
-      <c r="S35" s="123"/>
-      <c r="T35" s="123"/>
-      <c r="U35" s="114"/>
+      <c r="H35" s="124"/>
+      <c r="I35" s="124"/>
+      <c r="J35" s="124"/>
+      <c r="K35" s="124"/>
+      <c r="L35" s="124"/>
+      <c r="M35" s="124"/>
+      <c r="N35" s="124"/>
+      <c r="O35" s="124"/>
+      <c r="P35" s="124"/>
+      <c r="Q35" s="124"/>
+      <c r="R35" s="124"/>
+      <c r="S35" s="124"/>
+      <c r="T35" s="124"/>
+      <c r="U35" s="115"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="26"/>
-      <c r="B36" s="113" t="s">
+      <c r="A36" s="27"/>
+      <c r="B36" s="114" t="s">
+        <v>54</v>
+      </c>
+      <c r="C36" s="124"/>
+      <c r="U36" s="115"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="27"/>
+      <c r="B37" s="114"/>
+      <c r="C37" s="114"/>
+      <c r="D37" s="114"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="124"/>
+      <c r="I37" s="124"/>
+      <c r="J37" s="124"/>
+      <c r="K37" s="124"/>
+      <c r="L37" s="124"/>
+      <c r="M37" s="124"/>
+      <c r="N37" s="124"/>
+      <c r="O37" s="124"/>
+      <c r="P37" s="124"/>
+      <c r="Q37" s="124"/>
+      <c r="R37" s="124"/>
+      <c r="S37" s="124"/>
+      <c r="T37" s="124"/>
+      <c r="U37" s="115"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="27"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="28"/>
+      <c r="I38" s="28"/>
+      <c r="J38" s="28"/>
+      <c r="K38" s="28"/>
+      <c r="L38" s="28"/>
+      <c r="M38" s="28"/>
+      <c r="N38" s="28"/>
+      <c r="O38" s="28"/>
+      <c r="P38" s="28"/>
+      <c r="Q38" s="28"/>
+      <c r="R38" s="28"/>
+      <c r="S38" s="28"/>
+      <c r="T38" s="28"/>
+      <c r="U38" s="115"/>
+    </row>
+    <row r="39" ht="19.5" customHeight="1">
+      <c r="A39" s="125" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="123"/>
-      <c r="U36" s="114"/>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="26"/>
-      <c r="B37" s="113"/>
-      <c r="C37" s="113"/>
-      <c r="D37" s="113"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="29"/>
-      <c r="H37" s="123"/>
-      <c r="I37" s="123"/>
-      <c r="J37" s="123"/>
-      <c r="K37" s="123"/>
-      <c r="L37" s="123"/>
-      <c r="M37" s="123"/>
-      <c r="N37" s="123"/>
-      <c r="O37" s="123"/>
-      <c r="P37" s="123"/>
-      <c r="Q37" s="123"/>
-      <c r="R37" s="123"/>
-      <c r="S37" s="123"/>
-      <c r="T37" s="123"/>
-      <c r="U37" s="114"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="26"/>
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
-      <c r="J38" s="27"/>
-      <c r="K38" s="27"/>
-      <c r="L38" s="27"/>
-      <c r="M38" s="27"/>
-      <c r="N38" s="27"/>
-      <c r="O38" s="27"/>
-      <c r="P38" s="27"/>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="114"/>
-    </row>
-    <row r="39" ht="19.5" customHeight="1">
-      <c r="A39" s="124" t="s">
+      <c r="D39" s="28"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="126" t="s">
         <v>56</v>
       </c>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="125" t="s">
+      <c r="J39" s="28"/>
+      <c r="K39" s="126" t="s">
         <v>57</v>
       </c>
-      <c r="J39" s="27"/>
-      <c r="K39" s="125" t="s">
+      <c r="N39" s="28"/>
+      <c r="O39" s="28"/>
+      <c r="P39" s="126" t="s">
         <v>58</v>
       </c>
-      <c r="N39" s="27"/>
-      <c r="O39" s="27"/>
-      <c r="P39" s="125" t="s">
+      <c r="Q39" s="28"/>
+      <c r="R39" s="126" t="s">
         <v>59</v>
-      </c>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="125" t="s">
-        <v>60</v>
       </c>
       <c r="U39" s="11"/>
     </row>
     <row r="40" ht="19.5" customHeight="1">
       <c r="A40" s="10"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="J40" s="27"/>
-      <c r="N40" s="27"/>
-      <c r="O40" s="27"/>
-      <c r="Q40" s="27"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="J40" s="28"/>
+      <c r="N40" s="28"/>
+      <c r="O40" s="28"/>
+      <c r="Q40" s="28"/>
       <c r="U40" s="11"/>
     </row>
     <row r="41" ht="19.5" customHeight="1">
-      <c r="A41" s="126"/>
-      <c r="B41" s="120"/>
-      <c r="C41" s="120"/>
-      <c r="D41" s="127"/>
-      <c r="E41" s="127"/>
-      <c r="F41" s="120"/>
-      <c r="G41" s="120"/>
-      <c r="H41" s="120"/>
-      <c r="I41" s="120"/>
-      <c r="J41" s="127"/>
-      <c r="K41" s="120"/>
-      <c r="L41" s="120"/>
-      <c r="M41" s="120"/>
-      <c r="N41" s="127"/>
-      <c r="O41" s="127"/>
-      <c r="P41" s="120"/>
-      <c r="Q41" s="127"/>
-      <c r="R41" s="120"/>
-      <c r="S41" s="120"/>
-      <c r="T41" s="120"/>
+      <c r="A41" s="127"/>
+      <c r="B41" s="121"/>
+      <c r="C41" s="121"/>
+      <c r="D41" s="128"/>
+      <c r="E41" s="128"/>
+      <c r="F41" s="121"/>
+      <c r="G41" s="121"/>
+      <c r="H41" s="121"/>
+      <c r="I41" s="121"/>
+      <c r="J41" s="128"/>
+      <c r="K41" s="121"/>
+      <c r="L41" s="121"/>
+      <c r="M41" s="121"/>
+      <c r="N41" s="128"/>
+      <c r="O41" s="128"/>
+      <c r="P41" s="121"/>
+      <c r="Q41" s="128"/>
+      <c r="R41" s="121"/>
+      <c r="S41" s="121"/>
+      <c r="T41" s="121"/>
       <c r="U41" s="42"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="128"/>
+      <c r="A42" s="129"/>
     </row>
     <row r="43" ht="15.75" customHeight="1"/>
     <row r="44" ht="15.75" customHeight="1"/>
@@ -3615,9 +3554,11 @@
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="O10:P10"/>
-    <mergeCell ref="Q14:T14"/>
-    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="R19:T19"/>
+    <mergeCell ref="J24:M24"/>
+    <mergeCell ref="Q24:T24"/>
+    <mergeCell ref="K27:M27"/>
+    <mergeCell ref="R27:T27"/>
     <mergeCell ref="K28:M28"/>
     <mergeCell ref="R28:T28"/>
     <mergeCell ref="K29:M29"/>
@@ -3630,15 +3571,13 @@
     <mergeCell ref="P39:P41"/>
     <mergeCell ref="R39:U41"/>
     <mergeCell ref="A42:U43"/>
-    <mergeCell ref="K26:M26"/>
-    <mergeCell ref="K27:M27"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="G5:M5"/>
     <mergeCell ref="N5:Q5"/>
-    <mergeCell ref="C6:F6"/>
     <mergeCell ref="T6:U6"/>
+    <mergeCell ref="A7:F34"/>
     <mergeCell ref="J7:M7"/>
-    <mergeCell ref="A7:F34"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="A1:A4"/>
     <mergeCell ref="B1:D4"/>
     <mergeCell ref="E1:P4"/>
@@ -3650,14 +3589,14 @@
     <mergeCell ref="O7:P7"/>
     <mergeCell ref="O8:P8"/>
     <mergeCell ref="O9:P9"/>
+    <mergeCell ref="O10:P10"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="Q14:T14"/>
     <mergeCell ref="R16:T16"/>
     <mergeCell ref="R17:T17"/>
     <mergeCell ref="R18:T18"/>
-    <mergeCell ref="R19:T19"/>
-    <mergeCell ref="J24:M24"/>
-    <mergeCell ref="Q24:T24"/>
+    <mergeCell ref="K26:M26"/>
     <mergeCell ref="R26:T26"/>
-    <mergeCell ref="R27:T27"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins bottom="0.0" footer="0.0" header="0.0" left="0.0" right="0.0" top="0.393700787401575"/>

</xml_diff>

<commit_message>
feat: add configurable sheet cutting export header
</commit_message>
<xml_diff>
--- a/sheet_cutting_layout/templates/iatf/sheet_cutting_layout.xlsx
+++ b/sheet_cutting_layout/templates/iatf/sheet_cutting_layout.xlsx
@@ -19,16 +19,16 @@
     <t>TRIKAYA COATINGS Pvt. Ltd. Nashik</t>
   </si>
   <si>
-    <t>DOC. NO.:  FRM/PRD/15</t>
-  </si>
-  <si>
-    <t>REV. NO.: 01</t>
-  </si>
-  <si>
-    <t>REV DATE.: 03.07.2022</t>
-  </si>
-  <si>
-    <t>PAGE: 01 OF 01</t>
+    <t xml:space="preserve">DOC. NO.: </t>
+  </si>
+  <si>
+    <t>REV. NO.:</t>
+  </si>
+  <si>
+    <t>REV DATE.:</t>
+  </si>
+  <si>
+    <t>PAGE:</t>
   </si>
   <si>
     <t>Sheet Cutting Layout No:-</t>
@@ -816,7 +816,7 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -824,13 +824,13 @@
     <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="11" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="13" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="15" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="16" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="17" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -1126,36 +1126,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="504825" cy="504825"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr descr="TrikayaLogo.png" id="0" name="image1.png"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3574,10 +3545,10 @@
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="G5:M5"/>
     <mergeCell ref="N5:Q5"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="T6:U6"/>
     <mergeCell ref="A7:F34"/>
     <mergeCell ref="J7:M7"/>
-    <mergeCell ref="B6:F6"/>
     <mergeCell ref="A1:A4"/>
     <mergeCell ref="B1:D4"/>
     <mergeCell ref="E1:P4"/>

</xml_diff>